<commit_message>
rm ext dupl 5d55217e67877d71e36a079fa0146e2506f7f5fa
</commit_message>
<xml_diff>
--- a/nr-update-Organization-type/ig/StructureDefinition-as-ext-patient-type.xlsx
+++ b/nr-update-Organization-type/ig/StructureDefinition-as-ext-patient-type.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-20T16:47:04+00:00</t>
+    <t>2024-02-26T16:15:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -322,10 +322,10 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>Extension.extension:AuthorizedAgeRange</t>
-  </si>
-  <si>
-    <t>AuthorizedAgeRange</t>
+    <t>Extension.extension:authorizedAgeRange</t>
+  </si>
+  <si>
+    <t>authorizedAgeRange</t>
   </si>
   <si>
     <t>Age de la clientèle autorisée.</t>
@@ -334,19 +334,19 @@
     <t>An Extension</t>
   </si>
   <si>
-    <t>Extension.extension:AuthorizedAgeRange.id</t>
+    <t>Extension.extension:authorizedAgeRange.id</t>
   </si>
   <si>
     <t>Extension.extension.id</t>
   </si>
   <si>
-    <t>Extension.extension:AuthorizedAgeRange.extension</t>
+    <t>Extension.extension:authorizedAgeRange.extension</t>
   </si>
   <si>
     <t>Extension.extension.extension</t>
   </si>
   <si>
-    <t>Extension.extension:AuthorizedAgeRange.url</t>
+    <t>Extension.extension:authorizedAgeRange.url</t>
   </si>
   <si>
     <t>Extension.extension.url</t>
@@ -368,7 +368,7 @@
     <t>Extension.url</t>
   </si>
   <si>
-    <t>Extension.extension:AuthorizedAgeRange.value[x]</t>
+    <t>Extension.extension:authorizedAgeRange.value[x]</t>
   </si>
   <si>
     <t>Extension.extension.value[x]</t>
@@ -391,25 +391,25 @@
 </t>
   </si>
   <si>
-    <t>Extension.extension:InstalledAgeRange</t>
-  </si>
-  <si>
-    <t>InstalledAgeRange</t>
+    <t>Extension.extension:installedAgeRange</t>
+  </si>
+  <si>
+    <t>installedAgeRange</t>
   </si>
   <si>
     <t>Age de la clientèle installée.</t>
   </si>
   <si>
-    <t>Extension.extension:InstalledAgeRange.id</t>
-  </si>
-  <si>
-    <t>Extension.extension:InstalledAgeRange.extension</t>
-  </si>
-  <si>
-    <t>Extension.extension:InstalledAgeRange.url</t>
-  </si>
-  <si>
-    <t>Extension.extension:InstalledAgeRange.value[x]</t>
+    <t>Extension.extension:installedAgeRange.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:installedAgeRange.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:installedAgeRange.url</t>
+  </si>
+  <si>
+    <t>Extension.extension:installedAgeRange.value[x]</t>
   </si>
   <si>
     <t>base64Binary
@@ -726,9 +726,9 @@
   <dimension ref="A1:AK16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="49.09765625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="48.96875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="29.1484375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="20.375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="20.24609375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="12.64453125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.9453125" customWidth="true" bestFit="true"/>

</xml_diff>